<commit_message>
Update sample xlsx file
</commit_message>
<xml_diff>
--- a/26.02월 활동계획서 000반-이용자1 이용자2 이용자3-샘플.xlsx
+++ b/26.02월 활동계획서 000반-이용자1 이용자2 이용자3-샘플.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Untitled/계획서/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vintage_playlab/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B806A026-A5C8-E743-BC4A-45A83200F407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14058D6-4351-EE44-AD10-A425F2328264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="27880" windowHeight="17400" tabRatio="800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="27880" windowHeight="17400" tabRatio="800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="02월 계획서-유정빈" sheetId="10" r:id="rId1"/>
-    <sheet name="02월 계획서-모민준" sheetId="11" r:id="rId2"/>
-    <sheet name="02월 계획서-박소연" sheetId="8" r:id="rId3"/>
+    <sheet name="02월 계획서-이용자1" sheetId="10" r:id="rId1"/>
+    <sheet name="02월 계획서-이용자2" sheetId="11" r:id="rId2"/>
+    <sheet name="02월 계획서-이용자3" sheetId="8" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1303,6 +1303,87 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1312,242 +1393,161 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="3" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1858,176 +1858,176 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="50" customHeight="1">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="80"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="53"/>
+      <c r="N1" s="53"/>
+      <c r="O1" s="54"/>
     </row>
     <row r="2" spans="1:15" ht="30" customHeight="1">
       <c r="A2" s="55" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="56"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="81" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81" t="s">
+      <c r="E2" s="41"/>
+      <c r="F2" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81" t="s">
+      <c r="G2" s="41"/>
+      <c r="H2" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="I2" s="81"/>
-      <c r="J2" s="82"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="31"/>
       <c r="K2" s="56"/>
       <c r="L2" s="56"/>
       <c r="M2" s="56"/>
       <c r="N2" s="56"/>
-      <c r="O2" s="83"/>
+      <c r="O2" s="32"/>
     </row>
     <row r="3" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="65" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="65"/>
-      <c r="F3" s="61" t="s">
+      <c r="E3" s="64"/>
+      <c r="F3" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="61"/>
-      <c r="J3" s="95" t="s">
+      <c r="I3" s="33"/>
+      <c r="J3" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="60"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-      <c r="N3" s="59"/>
-      <c r="O3" s="94"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="30"/>
     </row>
     <row r="4" spans="1:15" ht="30" customHeight="1">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="72" t="s">
+      <c r="B4" s="66"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="71" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="73"/>
-      <c r="F4" s="76" t="s">
+      <c r="E4" s="72"/>
+      <c r="F4" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="77"/>
-      <c r="H4" s="52" t="s">
+      <c r="G4" s="76"/>
+      <c r="H4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="53"/>
-      <c r="J4" s="54">
+      <c r="I4" s="58"/>
+      <c r="J4" s="59">
         <f>SUM(L9:L25)</f>
         <v>0</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="L4" s="96" t="e">
+      <c r="K4" s="59"/>
+      <c r="L4" s="35" t="e">
         <f>J4/$F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="M4" s="97"/>
-      <c r="N4" s="97"/>
-      <c r="O4" s="98"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="37"/>
     </row>
     <row r="5" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A5" s="69"/>
-      <c r="B5" s="70"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="99">
+      <c r="A5" s="68"/>
+      <c r="B5" s="69"/>
+      <c r="C5" s="70"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="38">
         <f>SUM(L26:O26)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="100"/>
-      <c r="H5" s="57" t="s">
+      <c r="G5" s="39"/>
+      <c r="H5" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81">
+      <c r="I5" s="41"/>
+      <c r="J5" s="41">
         <f>SUM(M9:M25)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="81"/>
-      <c r="L5" s="101" t="e">
+      <c r="K5" s="41"/>
+      <c r="L5" s="42" t="e">
         <f t="shared" ref="L5:L7" si="0">J5/$F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="M5" s="102"/>
-      <c r="N5" s="102"/>
-      <c r="O5" s="103"/>
+      <c r="M5" s="43"/>
+      <c r="N5" s="43"/>
+      <c r="O5" s="44"/>
     </row>
     <row r="6" spans="1:15" ht="30" customHeight="1">
       <c r="A6" s="55" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="56"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="82" t="s">
+      <c r="C6" s="40"/>
+      <c r="D6" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="83"/>
+      <c r="E6" s="32"/>
       <c r="F6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="57" t="s">
+      <c r="H6" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="81"/>
-      <c r="J6" s="81">
+      <c r="I6" s="41"/>
+      <c r="J6" s="41">
         <f>SUM(N9:N25)</f>
         <v>0</v>
       </c>
-      <c r="K6" s="81"/>
-      <c r="L6" s="101" t="e">
+      <c r="K6" s="41"/>
+      <c r="L6" s="42" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="M6" s="102"/>
-      <c r="N6" s="102"/>
-      <c r="O6" s="103"/>
+      <c r="M6" s="43"/>
+      <c r="N6" s="43"/>
+      <c r="O6" s="44"/>
     </row>
     <row r="7" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="59"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="92"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="26"/>
       <c r="F7" s="4">
         <f>SUM(J4:K6)</f>
         <v>0</v>
@@ -2036,22 +2036,22 @@
         <f>SUM(J7)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="60" t="s">
+      <c r="H7" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="93"/>
-      <c r="J7" s="93">
+      <c r="I7" s="28"/>
+      <c r="J7" s="28">
         <f>SUM(O9:O25)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="93"/>
-      <c r="L7" s="88" t="e">
+      <c r="K7" s="28"/>
+      <c r="L7" s="22" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="M7" s="89"/>
-      <c r="N7" s="89"/>
-      <c r="O7" s="90"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="24"/>
     </row>
     <row r="8" spans="1:15" ht="38.25" customHeight="1">
       <c r="A8" s="6" t="s">
@@ -2063,20 +2063,20 @@
       <c r="C8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="84" t="s">
+      <c r="D8" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="85"/>
-      <c r="F8" s="86"/>
-      <c r="G8" s="87" t="s">
+      <c r="E8" s="46"/>
+      <c r="F8" s="47"/>
+      <c r="G8" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="87"/>
-      <c r="I8" s="87"/>
-      <c r="J8" s="85" t="s">
+      <c r="H8" s="48"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="86"/>
+      <c r="K8" s="47"/>
       <c r="L8" s="9" t="s">
         <v>10</v>
       </c>
@@ -2094,14 +2094,14 @@
       <c r="A9" s="18"/>
       <c r="B9" s="19"/>
       <c r="C9" s="12"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="24"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="49"/>
+      <c r="K9" s="51"/>
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
       <c r="N9" s="11"/>
@@ -2111,14 +2111,14 @@
       <c r="A10" s="18"/>
       <c r="B10" s="19"/>
       <c r="C10" s="12"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="48"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="50"/>
+      <c r="I10" s="51"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="77"/>
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
       <c r="N10" s="11"/>
@@ -2128,14 +2128,14 @@
       <c r="A11" s="18"/>
       <c r="B11" s="19"/>
       <c r="C11" s="12"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="48"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="78"/>
+      <c r="H11" s="79"/>
+      <c r="I11" s="80"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="77"/>
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
       <c r="N11" s="11"/>
@@ -2145,14 +2145,14 @@
       <c r="A12" s="18"/>
       <c r="B12" s="19"/>
       <c r="C12" s="12"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="48"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="51"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="50"/>
+      <c r="I12" s="51"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="77"/>
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
       <c r="N12" s="11"/>
@@ -2162,14 +2162,14 @@
       <c r="A13" s="18"/>
       <c r="B13" s="19"/>
       <c r="C13" s="12"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="50"/>
-      <c r="H13" s="51"/>
-      <c r="I13" s="48"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="82"/>
+      <c r="H13" s="83"/>
+      <c r="I13" s="77"/>
+      <c r="J13" s="49"/>
+      <c r="K13" s="81"/>
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
       <c r="N13" s="11"/>
@@ -2179,14 +2179,14 @@
       <c r="A14" s="18"/>
       <c r="B14" s="19"/>
       <c r="C14" s="12"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="48"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="78"/>
+      <c r="H14" s="79"/>
+      <c r="I14" s="80"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="77"/>
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
       <c r="N14" s="11"/>
@@ -2196,14 +2196,14 @@
       <c r="A15" s="18"/>
       <c r="B15" s="19"/>
       <c r="C15" s="12"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="48"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="51"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="77"/>
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
       <c r="N15" s="11"/>
@@ -2213,14 +2213,14 @@
       <c r="A16" s="18"/>
       <c r="B16" s="19"/>
       <c r="C16" s="12"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="24"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="48"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="50"/>
+      <c r="I16" s="51"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="77"/>
       <c r="L16" s="11"/>
       <c r="M16" s="11"/>
       <c r="N16" s="11"/>
@@ -2230,14 +2230,14 @@
       <c r="A17" s="18"/>
       <c r="B17" s="19"/>
       <c r="C17" s="12"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="24"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="48"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="77"/>
       <c r="L17" s="11"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
@@ -2247,14 +2247,14 @@
       <c r="A18" s="18"/>
       <c r="B18" s="19"/>
       <c r="C18" s="12"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="24"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="49"/>
+      <c r="K18" s="51"/>
       <c r="L18" s="11"/>
       <c r="M18" s="11"/>
       <c r="N18" s="11"/>
@@ -2264,14 +2264,14 @@
       <c r="A19" s="18"/>
       <c r="B19" s="19"/>
       <c r="C19" s="12"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="48"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="49"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="77"/>
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>
       <c r="N19" s="11"/>
@@ -2281,14 +2281,14 @@
       <c r="A20" s="18"/>
       <c r="B20" s="19"/>
       <c r="C20" s="12"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="24"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="51"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="51"/>
       <c r="L20" s="11"/>
       <c r="M20" s="11"/>
       <c r="N20" s="11"/>
@@ -2298,14 +2298,14 @@
       <c r="A21" s="18"/>
       <c r="B21" s="19"/>
       <c r="C21" s="12"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="24"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="51"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="51"/>
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
       <c r="N21" s="11"/>
@@ -2315,14 +2315,14 @@
       <c r="A22" s="18"/>
       <c r="B22" s="19"/>
       <c r="C22" s="12"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="29"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="29"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="78"/>
+      <c r="H22" s="79"/>
+      <c r="I22" s="80"/>
+      <c r="J22" s="78"/>
+      <c r="K22" s="80"/>
       <c r="L22" s="11"/>
       <c r="M22" s="11"/>
       <c r="N22" s="11"/>
@@ -2332,14 +2332,14 @@
       <c r="A23" s="18"/>
       <c r="B23" s="19"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="48"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="50"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="77"/>
       <c r="L23" s="11"/>
       <c r="M23" s="11"/>
       <c r="N23" s="11"/>
@@ -2349,14 +2349,14 @@
       <c r="A24" s="18"/>
       <c r="B24" s="19"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="23"/>
-      <c r="I24" s="24"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="26"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="102"/>
+      <c r="K24" s="103"/>
       <c r="L24" s="11"/>
       <c r="M24" s="11"/>
       <c r="N24" s="11"/>
@@ -2366,12 +2366,12 @@
       <c r="A25" s="18"/>
       <c r="B25" s="19"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="29"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="79"/>
+      <c r="I25" s="80"/>
       <c r="J25" s="20"/>
       <c r="K25" s="21"/>
       <c r="L25" s="11"/>
@@ -2380,19 +2380,19 @@
       <c r="O25" s="13"/>
     </row>
     <row r="26" spans="1:15" ht="27.5" customHeight="1" thickBot="1">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="35"/>
+      <c r="B26" s="88"/>
+      <c r="C26" s="88"/>
+      <c r="D26" s="88"/>
+      <c r="E26" s="88"/>
+      <c r="F26" s="88"/>
+      <c r="G26" s="88"/>
+      <c r="H26" s="88"/>
+      <c r="I26" s="88"/>
+      <c r="J26" s="88"/>
+      <c r="K26" s="89"/>
       <c r="L26" s="14">
         <f>SUM(L9:L25)</f>
         <v>0</v>
@@ -2411,102 +2411,178 @@
       </c>
     </row>
     <row r="27" spans="1:15" ht="99.5" customHeight="1" thickBot="1">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="90" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="39" t="s">
+      <c r="B27" s="91"/>
+      <c r="C27" s="92"/>
+      <c r="D27" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="40"/>
-      <c r="J27" s="40"/>
-      <c r="K27" s="40"/>
-      <c r="L27" s="40"/>
-      <c r="M27" s="40"/>
-      <c r="N27" s="40"/>
-      <c r="O27" s="41"/>
+      <c r="E27" s="94"/>
+      <c r="F27" s="94"/>
+      <c r="G27" s="94"/>
+      <c r="H27" s="94"/>
+      <c r="I27" s="94"/>
+      <c r="J27" s="94"/>
+      <c r="K27" s="94"/>
+      <c r="L27" s="94"/>
+      <c r="M27" s="94"/>
+      <c r="N27" s="94"/>
+      <c r="O27" s="95"/>
     </row>
     <row r="28" spans="1:15" ht="44" customHeight="1">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="96" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="43"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="43"/>
-      <c r="I28" s="43"/>
-      <c r="J28" s="43"/>
-      <c r="K28" s="43"/>
-      <c r="L28" s="43"/>
-      <c r="M28" s="43"/>
-      <c r="N28" s="43"/>
-      <c r="O28" s="44"/>
+      <c r="B28" s="97"/>
+      <c r="C28" s="97"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="97"/>
+      <c r="G28" s="97"/>
+      <c r="H28" s="97"/>
+      <c r="I28" s="97"/>
+      <c r="J28" s="97"/>
+      <c r="K28" s="97"/>
+      <c r="L28" s="97"/>
+      <c r="M28" s="97"/>
+      <c r="N28" s="97"/>
+      <c r="O28" s="98"/>
     </row>
     <row r="29" spans="1:15" ht="59.75" customHeight="1">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="99" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="46"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46"/>
-      <c r="H29" s="46"/>
-      <c r="I29" s="46"/>
-      <c r="J29" s="46"/>
-      <c r="K29" s="46"/>
-      <c r="L29" s="46"/>
-      <c r="M29" s="46"/>
-      <c r="N29" s="46"/>
-      <c r="O29" s="47"/>
+      <c r="B29" s="100"/>
+      <c r="C29" s="100"/>
+      <c r="D29" s="100"/>
+      <c r="E29" s="100"/>
+      <c r="F29" s="100"/>
+      <c r="G29" s="100"/>
+      <c r="H29" s="100"/>
+      <c r="I29" s="100"/>
+      <c r="J29" s="100"/>
+      <c r="K29" s="100"/>
+      <c r="L29" s="100"/>
+      <c r="M29" s="100"/>
+      <c r="N29" s="100"/>
+      <c r="O29" s="101"/>
     </row>
     <row r="30" spans="1:15" ht="62" customHeight="1">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="99" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="46"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="46"/>
-      <c r="J30" s="46"/>
-      <c r="K30" s="46"/>
-      <c r="L30" s="46"/>
-      <c r="M30" s="46"/>
-      <c r="N30" s="46"/>
-      <c r="O30" s="47"/>
+      <c r="B30" s="100"/>
+      <c r="C30" s="100"/>
+      <c r="D30" s="100"/>
+      <c r="E30" s="100"/>
+      <c r="F30" s="100"/>
+      <c r="G30" s="100"/>
+      <c r="H30" s="100"/>
+      <c r="I30" s="100"/>
+      <c r="J30" s="100"/>
+      <c r="K30" s="100"/>
+      <c r="L30" s="100"/>
+      <c r="M30" s="100"/>
+      <c r="N30" s="100"/>
+      <c r="O30" s="101"/>
     </row>
     <row r="31" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A31" s="30"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
-      <c r="J31" s="31"/>
-      <c r="K31" s="31"/>
-      <c r="L31" s="31"/>
-      <c r="M31" s="31"/>
-      <c r="N31" s="31"/>
-      <c r="O31" s="32"/>
+      <c r="A31" s="84"/>
+      <c r="B31" s="85"/>
+      <c r="C31" s="85"/>
+      <c r="D31" s="85"/>
+      <c r="E31" s="85"/>
+      <c r="F31" s="85"/>
+      <c r="G31" s="85"/>
+      <c r="H31" s="85"/>
+      <c r="I31" s="85"/>
+      <c r="J31" s="85"/>
+      <c r="K31" s="85"/>
+      <c r="L31" s="85"/>
+      <c r="M31" s="85"/>
+      <c r="N31" s="85"/>
+      <c r="O31" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="92">
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="A31:O31"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:O27"/>
+    <mergeCell ref="A28:O28"/>
+    <mergeCell ref="A29:O29"/>
+    <mergeCell ref="A30:O30"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="A4:C5"/>
+    <mergeCell ref="D4:E5"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:O2"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:K9"/>
     <mergeCell ref="L7:O7"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="H7:I7"/>
@@ -2523,82 +2599,6 @@
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="L6:O6"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:O2"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="A4:C5"/>
-    <mergeCell ref="D4:E5"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="A31:O31"/>
-    <mergeCell ref="A26:K26"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="D27:O27"/>
-    <mergeCell ref="A28:O28"/>
-    <mergeCell ref="A29:O29"/>
-    <mergeCell ref="A30:O30"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="G25:I25"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
@@ -2637,176 +2637,176 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="50" customHeight="1">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="80"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="53"/>
+      <c r="N1" s="53"/>
+      <c r="O1" s="54"/>
     </row>
     <row r="2" spans="1:15" ht="30" customHeight="1">
       <c r="A2" s="55" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="56"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="81" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81" t="s">
+      <c r="E2" s="41"/>
+      <c r="F2" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81" t="s">
+      <c r="G2" s="41"/>
+      <c r="H2" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="I2" s="81"/>
-      <c r="J2" s="82"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="31"/>
       <c r="K2" s="56"/>
       <c r="L2" s="56"/>
       <c r="M2" s="56"/>
       <c r="N2" s="56"/>
-      <c r="O2" s="83"/>
+      <c r="O2" s="32"/>
     </row>
     <row r="3" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="65" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="65"/>
-      <c r="F3" s="61" t="s">
+      <c r="E3" s="64"/>
+      <c r="F3" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="61"/>
-      <c r="J3" s="95" t="s">
+      <c r="I3" s="33"/>
+      <c r="J3" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="60"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-      <c r="N3" s="59"/>
-      <c r="O3" s="94"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="30"/>
     </row>
     <row r="4" spans="1:15" ht="30" customHeight="1">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="72" t="s">
+      <c r="B4" s="66"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="71" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="73"/>
-      <c r="F4" s="76" t="s">
+      <c r="E4" s="72"/>
+      <c r="F4" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="77"/>
-      <c r="H4" s="52" t="s">
+      <c r="G4" s="76"/>
+      <c r="H4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="53"/>
-      <c r="J4" s="54">
+      <c r="I4" s="58"/>
+      <c r="J4" s="59">
         <f>SUM(L9:L25)</f>
         <v>0</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="L4" s="96" t="e">
+      <c r="K4" s="59"/>
+      <c r="L4" s="35" t="e">
         <f>J4/$F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="M4" s="97"/>
-      <c r="N4" s="97"/>
-      <c r="O4" s="98"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="37"/>
     </row>
     <row r="5" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A5" s="69"/>
-      <c r="B5" s="70"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="99">
+      <c r="A5" s="68"/>
+      <c r="B5" s="69"/>
+      <c r="C5" s="70"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="38">
         <f>SUM(L26:O26)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="100"/>
-      <c r="H5" s="57" t="s">
+      <c r="G5" s="39"/>
+      <c r="H5" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81">
+      <c r="I5" s="41"/>
+      <c r="J5" s="41">
         <f>SUM(M9:M25)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="81"/>
-      <c r="L5" s="101" t="e">
+      <c r="K5" s="41"/>
+      <c r="L5" s="42" t="e">
         <f t="shared" ref="L5:L7" si="0">J5/$F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="M5" s="102"/>
-      <c r="N5" s="102"/>
-      <c r="O5" s="103"/>
+      <c r="M5" s="43"/>
+      <c r="N5" s="43"/>
+      <c r="O5" s="44"/>
     </row>
     <row r="6" spans="1:15" ht="30" customHeight="1">
       <c r="A6" s="55" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="56"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="82" t="s">
+      <c r="C6" s="40"/>
+      <c r="D6" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="83"/>
+      <c r="E6" s="32"/>
       <c r="F6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="57" t="s">
+      <c r="H6" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="81"/>
-      <c r="J6" s="81">
+      <c r="I6" s="41"/>
+      <c r="J6" s="41">
         <f>SUM(N9:N25)</f>
         <v>0</v>
       </c>
-      <c r="K6" s="81"/>
-      <c r="L6" s="101" t="e">
+      <c r="K6" s="41"/>
+      <c r="L6" s="42" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="M6" s="102"/>
-      <c r="N6" s="102"/>
-      <c r="O6" s="103"/>
+      <c r="M6" s="43"/>
+      <c r="N6" s="43"/>
+      <c r="O6" s="44"/>
     </row>
     <row r="7" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="59"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="92"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="26"/>
       <c r="F7" s="4">
         <f>SUM(J4:K6)</f>
         <v>0</v>
@@ -2815,22 +2815,22 @@
         <f>SUM(J7)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="60" t="s">
+      <c r="H7" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="93"/>
-      <c r="J7" s="93">
+      <c r="I7" s="28"/>
+      <c r="J7" s="28">
         <f>SUM(O9:O25)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="93"/>
-      <c r="L7" s="88" t="e">
+      <c r="K7" s="28"/>
+      <c r="L7" s="22" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="M7" s="89"/>
-      <c r="N7" s="89"/>
-      <c r="O7" s="90"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="24"/>
     </row>
     <row r="8" spans="1:15" ht="38.25" customHeight="1">
       <c r="A8" s="6" t="s">
@@ -2842,20 +2842,20 @@
       <c r="C8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="84" t="s">
+      <c r="D8" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="85"/>
-      <c r="F8" s="86"/>
-      <c r="G8" s="87" t="s">
+      <c r="E8" s="46"/>
+      <c r="F8" s="47"/>
+      <c r="G8" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="87"/>
-      <c r="I8" s="87"/>
-      <c r="J8" s="85" t="s">
+      <c r="H8" s="48"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="86"/>
+      <c r="K8" s="47"/>
       <c r="L8" s="9" t="s">
         <v>10</v>
       </c>
@@ -2873,14 +2873,14 @@
       <c r="A9" s="18"/>
       <c r="B9" s="19"/>
       <c r="C9" s="12"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="24"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="49"/>
+      <c r="K9" s="51"/>
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
       <c r="N9" s="11"/>
@@ -2890,14 +2890,14 @@
       <c r="A10" s="18"/>
       <c r="B10" s="19"/>
       <c r="C10" s="12"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="24"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="50"/>
+      <c r="I10" s="51"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="51"/>
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
       <c r="N10" s="11"/>
@@ -2907,14 +2907,14 @@
       <c r="A11" s="18"/>
       <c r="B11" s="19"/>
       <c r="C11" s="12"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="24"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="50"/>
+      <c r="I11" s="51"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="51"/>
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
       <c r="N11" s="11"/>
@@ -2924,14 +2924,14 @@
       <c r="A12" s="18"/>
       <c r="B12" s="19"/>
       <c r="C12" s="12"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="29"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="48"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="51"/>
+      <c r="G12" s="78"/>
+      <c r="H12" s="79"/>
+      <c r="I12" s="80"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="77"/>
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
       <c r="N12" s="11"/>
@@ -2941,14 +2941,14 @@
       <c r="A13" s="18"/>
       <c r="B13" s="19"/>
       <c r="C13" s="12"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="24"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="49"/>
+      <c r="H13" s="50"/>
+      <c r="I13" s="51"/>
       <c r="J13" s="104"/>
-      <c r="K13" s="48"/>
+      <c r="K13" s="77"/>
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
       <c r="N13" s="11"/>
@@ -2958,14 +2958,14 @@
       <c r="A14" s="18"/>
       <c r="B14" s="19"/>
       <c r="C14" s="12"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="50"/>
-      <c r="H14" s="51"/>
-      <c r="I14" s="48"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="48"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="82"/>
+      <c r="H14" s="83"/>
+      <c r="I14" s="77"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="77"/>
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
       <c r="N14" s="11"/>
@@ -2975,14 +2975,14 @@
       <c r="A15" s="18"/>
       <c r="B15" s="19"/>
       <c r="C15" s="12"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="29"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="48"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="78"/>
+      <c r="H15" s="79"/>
+      <c r="I15" s="80"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="77"/>
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
       <c r="N15" s="11"/>
@@ -2992,14 +2992,14 @@
       <c r="A16" s="18"/>
       <c r="B16" s="19"/>
       <c r="C16" s="12"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="24"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="48"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="50"/>
+      <c r="I16" s="51"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="77"/>
       <c r="L16" s="11"/>
       <c r="M16" s="11"/>
       <c r="N16" s="11"/>
@@ -3009,14 +3009,14 @@
       <c r="A17" s="18"/>
       <c r="B17" s="19"/>
       <c r="C17" s="12"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="24"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="48"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="77"/>
       <c r="L17" s="11"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
@@ -3026,14 +3026,14 @@
       <c r="A18" s="18"/>
       <c r="B18" s="19"/>
       <c r="C18" s="12"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="48"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="49"/>
+      <c r="K18" s="77"/>
       <c r="L18" s="11"/>
       <c r="M18" s="11"/>
       <c r="N18" s="11"/>
@@ -3043,14 +3043,14 @@
       <c r="A19" s="18"/>
       <c r="B19" s="19"/>
       <c r="C19" s="12"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="48"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="49"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="77"/>
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>
       <c r="N19" s="11"/>
@@ -3060,14 +3060,14 @@
       <c r="A20" s="18"/>
       <c r="B20" s="19"/>
       <c r="C20" s="12"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="48"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="51"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="77"/>
       <c r="L20" s="11"/>
       <c r="M20" s="11"/>
       <c r="N20" s="11"/>
@@ -3077,14 +3077,14 @@
       <c r="A21" s="18"/>
       <c r="B21" s="19"/>
       <c r="C21" s="12"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="24"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="51"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="51"/>
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
       <c r="N21" s="11"/>
@@ -3094,14 +3094,14 @@
       <c r="A22" s="18"/>
       <c r="B22" s="19"/>
       <c r="C22" s="12"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="23"/>
-      <c r="I22" s="24"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="48"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="49"/>
+      <c r="K22" s="77"/>
       <c r="L22" s="11"/>
       <c r="M22" s="11"/>
       <c r="N22" s="11"/>
@@ -3111,14 +3111,14 @@
       <c r="A23" s="18"/>
       <c r="B23" s="19"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="29"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="29"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="79"/>
+      <c r="I23" s="80"/>
+      <c r="J23" s="78"/>
+      <c r="K23" s="80"/>
       <c r="L23" s="11"/>
       <c r="M23" s="11"/>
       <c r="N23" s="11"/>
@@ -3128,14 +3128,14 @@
       <c r="A24" s="18"/>
       <c r="B24" s="19"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="28"/>
-      <c r="I24" s="29"/>
-      <c r="J24" s="27"/>
-      <c r="K24" s="29"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="79"/>
+      <c r="I24" s="80"/>
+      <c r="J24" s="78"/>
+      <c r="K24" s="80"/>
       <c r="L24" s="11"/>
       <c r="M24" s="11"/>
       <c r="N24" s="11"/>
@@ -3145,33 +3145,33 @@
       <c r="A25" s="18"/>
       <c r="B25" s="19"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="27"/>
-      <c r="K25" s="29"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="79"/>
+      <c r="I25" s="80"/>
+      <c r="J25" s="78"/>
+      <c r="K25" s="80"/>
       <c r="L25" s="11"/>
       <c r="M25" s="11"/>
       <c r="N25" s="11"/>
       <c r="O25" s="13"/>
     </row>
     <row r="26" spans="1:15" ht="27.5" customHeight="1" thickBot="1">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="35"/>
+      <c r="B26" s="88"/>
+      <c r="C26" s="88"/>
+      <c r="D26" s="88"/>
+      <c r="E26" s="88"/>
+      <c r="F26" s="88"/>
+      <c r="G26" s="88"/>
+      <c r="H26" s="88"/>
+      <c r="I26" s="88"/>
+      <c r="J26" s="88"/>
+      <c r="K26" s="89"/>
       <c r="L26" s="14">
         <f>SUM(L9:L25)</f>
         <v>0</v>
@@ -3190,102 +3190,179 @@
       </c>
     </row>
     <row r="27" spans="1:15" ht="99.5" customHeight="1" thickBot="1">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="90" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="39" t="s">
+      <c r="B27" s="91"/>
+      <c r="C27" s="92"/>
+      <c r="D27" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="40"/>
-      <c r="J27" s="40"/>
-      <c r="K27" s="40"/>
-      <c r="L27" s="40"/>
-      <c r="M27" s="40"/>
-      <c r="N27" s="40"/>
-      <c r="O27" s="41"/>
+      <c r="E27" s="94"/>
+      <c r="F27" s="94"/>
+      <c r="G27" s="94"/>
+      <c r="H27" s="94"/>
+      <c r="I27" s="94"/>
+      <c r="J27" s="94"/>
+      <c r="K27" s="94"/>
+      <c r="L27" s="94"/>
+      <c r="M27" s="94"/>
+      <c r="N27" s="94"/>
+      <c r="O27" s="95"/>
     </row>
     <row r="28" spans="1:15" ht="44" customHeight="1">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="96" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="43"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="43"/>
-      <c r="I28" s="43"/>
-      <c r="J28" s="43"/>
-      <c r="K28" s="43"/>
-      <c r="L28" s="43"/>
-      <c r="M28" s="43"/>
-      <c r="N28" s="43"/>
-      <c r="O28" s="44"/>
+      <c r="B28" s="97"/>
+      <c r="C28" s="97"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="97"/>
+      <c r="G28" s="97"/>
+      <c r="H28" s="97"/>
+      <c r="I28" s="97"/>
+      <c r="J28" s="97"/>
+      <c r="K28" s="97"/>
+      <c r="L28" s="97"/>
+      <c r="M28" s="97"/>
+      <c r="N28" s="97"/>
+      <c r="O28" s="98"/>
     </row>
     <row r="29" spans="1:15" ht="68" customHeight="1">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="99" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="46"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46"/>
-      <c r="H29" s="46"/>
-      <c r="I29" s="46"/>
-      <c r="J29" s="46"/>
-      <c r="K29" s="46"/>
-      <c r="L29" s="46"/>
-      <c r="M29" s="46"/>
-      <c r="N29" s="46"/>
-      <c r="O29" s="47"/>
+      <c r="B29" s="100"/>
+      <c r="C29" s="100"/>
+      <c r="D29" s="100"/>
+      <c r="E29" s="100"/>
+      <c r="F29" s="100"/>
+      <c r="G29" s="100"/>
+      <c r="H29" s="100"/>
+      <c r="I29" s="100"/>
+      <c r="J29" s="100"/>
+      <c r="K29" s="100"/>
+      <c r="L29" s="100"/>
+      <c r="M29" s="100"/>
+      <c r="N29" s="100"/>
+      <c r="O29" s="101"/>
     </row>
     <row r="30" spans="1:15" ht="68" customHeight="1">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="99" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="46"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="46"/>
-      <c r="J30" s="46"/>
-      <c r="K30" s="46"/>
-      <c r="L30" s="46"/>
-      <c r="M30" s="46"/>
-      <c r="N30" s="46"/>
-      <c r="O30" s="47"/>
+      <c r="B30" s="100"/>
+      <c r="C30" s="100"/>
+      <c r="D30" s="100"/>
+      <c r="E30" s="100"/>
+      <c r="F30" s="100"/>
+      <c r="G30" s="100"/>
+      <c r="H30" s="100"/>
+      <c r="I30" s="100"/>
+      <c r="J30" s="100"/>
+      <c r="K30" s="100"/>
+      <c r="L30" s="100"/>
+      <c r="M30" s="100"/>
+      <c r="N30" s="100"/>
+      <c r="O30" s="101"/>
     </row>
     <row r="31" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A31" s="30"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
-      <c r="J31" s="31"/>
-      <c r="K31" s="31"/>
-      <c r="L31" s="31"/>
-      <c r="M31" s="31"/>
-      <c r="N31" s="31"/>
-      <c r="O31" s="32"/>
+      <c r="A31" s="84"/>
+      <c r="B31" s="85"/>
+      <c r="C31" s="85"/>
+      <c r="D31" s="85"/>
+      <c r="E31" s="85"/>
+      <c r="F31" s="85"/>
+      <c r="G31" s="85"/>
+      <c r="H31" s="85"/>
+      <c r="I31" s="85"/>
+      <c r="J31" s="85"/>
+      <c r="K31" s="85"/>
+      <c r="L31" s="85"/>
+      <c r="M31" s="85"/>
+      <c r="N31" s="85"/>
+      <c r="O31" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="93">
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L4:O4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="L3:O3"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:O5"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:O2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="L7:O7"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="A4:C5"/>
+    <mergeCell ref="D4:E5"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="D12:F12"/>
     <mergeCell ref="G25:I25"/>
     <mergeCell ref="J11:K11"/>
     <mergeCell ref="G11:I11"/>
@@ -3302,83 +3379,6 @@
     <mergeCell ref="G24:I24"/>
     <mergeCell ref="J24:K24"/>
     <mergeCell ref="J25:K25"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="A4:C5"/>
-    <mergeCell ref="D4:E5"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="L7:O7"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:O2"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L4:O4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="L3:O3"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:O5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
@@ -3418,176 +3418,176 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="50" customHeight="1">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="80"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="53"/>
+      <c r="N1" s="53"/>
+      <c r="O1" s="54"/>
     </row>
     <row r="2" spans="1:15" ht="30" customHeight="1">
       <c r="A2" s="55" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="56"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="81" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81" t="s">
+      <c r="E2" s="41"/>
+      <c r="F2" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81" t="s">
+      <c r="G2" s="41"/>
+      <c r="H2" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="I2" s="81"/>
-      <c r="J2" s="82"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="31"/>
       <c r="K2" s="56"/>
       <c r="L2" s="56"/>
       <c r="M2" s="56"/>
       <c r="N2" s="56"/>
-      <c r="O2" s="83"/>
+      <c r="O2" s="32"/>
     </row>
     <row r="3" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="65" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="64" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="65"/>
-      <c r="F3" s="61" t="s">
+      <c r="E3" s="64"/>
+      <c r="F3" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="61"/>
-      <c r="J3" s="95" t="s">
+      <c r="I3" s="33"/>
+      <c r="J3" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="60"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-      <c r="N3" s="59"/>
-      <c r="O3" s="94"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="30"/>
     </row>
     <row r="4" spans="1:15" ht="30" customHeight="1">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="72" t="s">
+      <c r="B4" s="66"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="71" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="73"/>
-      <c r="F4" s="76" t="s">
+      <c r="E4" s="72"/>
+      <c r="F4" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="77"/>
-      <c r="H4" s="52" t="s">
+      <c r="G4" s="76"/>
+      <c r="H4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="53"/>
-      <c r="J4" s="54">
+      <c r="I4" s="58"/>
+      <c r="J4" s="59">
         <f>SUM(L9:L25)</f>
         <v>0</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="L4" s="96" t="e">
+      <c r="K4" s="59"/>
+      <c r="L4" s="35" t="e">
         <f>J4/$F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="M4" s="97"/>
-      <c r="N4" s="97"/>
-      <c r="O4" s="98"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="37"/>
     </row>
     <row r="5" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A5" s="69"/>
-      <c r="B5" s="70"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="99">
+      <c r="A5" s="68"/>
+      <c r="B5" s="69"/>
+      <c r="C5" s="70"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="38">
         <f>SUM(L26:O26)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="100"/>
-      <c r="H5" s="57" t="s">
+      <c r="G5" s="39"/>
+      <c r="H5" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81">
+      <c r="I5" s="41"/>
+      <c r="J5" s="41">
         <f>SUM(M9:M25)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="81"/>
-      <c r="L5" s="101" t="e">
+      <c r="K5" s="41"/>
+      <c r="L5" s="42" t="e">
         <f t="shared" ref="L5:L7" si="0">J5/$F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="M5" s="102"/>
-      <c r="N5" s="102"/>
-      <c r="O5" s="103"/>
+      <c r="M5" s="43"/>
+      <c r="N5" s="43"/>
+      <c r="O5" s="44"/>
     </row>
     <row r="6" spans="1:15" ht="30" customHeight="1">
       <c r="A6" s="55" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="56"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="82" t="s">
+      <c r="C6" s="40"/>
+      <c r="D6" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="83"/>
+      <c r="E6" s="32"/>
       <c r="F6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="57" t="s">
+      <c r="H6" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="81"/>
-      <c r="J6" s="81">
+      <c r="I6" s="41"/>
+      <c r="J6" s="41">
         <f>SUM(N9:N25)</f>
         <v>0</v>
       </c>
-      <c r="K6" s="81"/>
-      <c r="L6" s="101" t="e">
+      <c r="K6" s="41"/>
+      <c r="L6" s="42" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="M6" s="102"/>
-      <c r="N6" s="102"/>
-      <c r="O6" s="103"/>
+      <c r="M6" s="43"/>
+      <c r="N6" s="43"/>
+      <c r="O6" s="44"/>
     </row>
     <row r="7" spans="1:15" ht="30" customHeight="1" thickBot="1">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="59"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="92"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="26"/>
       <c r="F7" s="4">
         <f>SUM(J4:K6)</f>
         <v>0</v>
@@ -3596,22 +3596,22 @@
         <f>SUM(J7)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="60" t="s">
+      <c r="H7" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="93"/>
-      <c r="J7" s="93">
+      <c r="I7" s="28"/>
+      <c r="J7" s="28">
         <f>SUM(O9:O25)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="93"/>
-      <c r="L7" s="88" t="e">
+      <c r="K7" s="28"/>
+      <c r="L7" s="22" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="M7" s="89"/>
-      <c r="N7" s="89"/>
-      <c r="O7" s="90"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="24"/>
     </row>
     <row r="8" spans="1:15" ht="38.25" customHeight="1">
       <c r="A8" s="6" t="s">
@@ -3623,20 +3623,20 @@
       <c r="C8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="84" t="s">
+      <c r="D8" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="85"/>
-      <c r="F8" s="86"/>
-      <c r="G8" s="87" t="s">
+      <c r="E8" s="46"/>
+      <c r="F8" s="47"/>
+      <c r="G8" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="87"/>
-      <c r="I8" s="87"/>
-      <c r="J8" s="85" t="s">
+      <c r="H8" s="48"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="46" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="86"/>
+      <c r="K8" s="47"/>
       <c r="L8" s="9" t="s">
         <v>10</v>
       </c>
@@ -3654,14 +3654,14 @@
       <c r="A9" s="18"/>
       <c r="B9" s="19"/>
       <c r="C9" s="12"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="24"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="49"/>
+      <c r="K9" s="51"/>
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
       <c r="N9" s="11"/>
@@ -3671,14 +3671,14 @@
       <c r="A10" s="18"/>
       <c r="B10" s="19"/>
       <c r="C10" s="12"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="24"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="50"/>
+      <c r="I10" s="51"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="51"/>
       <c r="L10" s="11"/>
       <c r="M10" s="11"/>
       <c r="N10" s="11"/>
@@ -3688,14 +3688,14 @@
       <c r="A11" s="18"/>
       <c r="B11" s="19"/>
       <c r="C11" s="12"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="24"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="50"/>
+      <c r="I11" s="51"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="51"/>
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
       <c r="N11" s="11"/>
@@ -3705,14 +3705,14 @@
       <c r="A12" s="18"/>
       <c r="B12" s="19"/>
       <c r="C12" s="12"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="24"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="51"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="50"/>
+      <c r="I12" s="51"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="51"/>
       <c r="L12" s="11"/>
       <c r="M12" s="11"/>
       <c r="N12" s="11"/>
@@ -3722,14 +3722,14 @@
       <c r="A13" s="18"/>
       <c r="B13" s="19"/>
       <c r="C13" s="12"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="24"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="49"/>
+      <c r="H13" s="50"/>
+      <c r="I13" s="51"/>
+      <c r="J13" s="49"/>
+      <c r="K13" s="51"/>
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
       <c r="N13" s="11"/>
@@ -3739,14 +3739,14 @@
       <c r="A14" s="18"/>
       <c r="B14" s="19"/>
       <c r="C14" s="12"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="24"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="78"/>
+      <c r="H14" s="79"/>
+      <c r="I14" s="80"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="51"/>
       <c r="L14" s="11"/>
       <c r="M14" s="11"/>
       <c r="N14" s="11"/>
@@ -3756,14 +3756,14 @@
       <c r="A15" s="18"/>
       <c r="B15" s="19"/>
       <c r="C15" s="12"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="24"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="51"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="51"/>
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
       <c r="N15" s="11"/>
@@ -3773,14 +3773,14 @@
       <c r="A16" s="18"/>
       <c r="B16" s="19"/>
       <c r="C16" s="12"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="50"/>
-      <c r="H16" s="51"/>
-      <c r="I16" s="48"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="24"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="82"/>
+      <c r="H16" s="83"/>
+      <c r="I16" s="77"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="51"/>
       <c r="L16" s="11"/>
       <c r="M16" s="11"/>
       <c r="N16" s="11"/>
@@ -3790,14 +3790,14 @@
       <c r="A17" s="18"/>
       <c r="B17" s="19"/>
       <c r="C17" s="12"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="29"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="24"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="78"/>
+      <c r="H17" s="79"/>
+      <c r="I17" s="80"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="51"/>
       <c r="L17" s="11"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
@@ -3807,14 +3807,14 @@
       <c r="A18" s="18"/>
       <c r="B18" s="19"/>
       <c r="C18" s="12"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="24"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="49"/>
+      <c r="K18" s="51"/>
       <c r="L18" s="11"/>
       <c r="M18" s="11"/>
       <c r="N18" s="11"/>
@@ -3824,14 +3824,14 @@
       <c r="A19" s="18"/>
       <c r="B19" s="19"/>
       <c r="C19" s="12"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="24"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="49"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="51"/>
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>
       <c r="N19" s="11"/>
@@ -3841,14 +3841,14 @@
       <c r="A20" s="18"/>
       <c r="B20" s="19"/>
       <c r="C20" s="12"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="24"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="51"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="51"/>
       <c r="L20" s="11"/>
       <c r="M20" s="11"/>
       <c r="N20" s="11"/>
@@ -3858,14 +3858,14 @@
       <c r="A21" s="18"/>
       <c r="B21" s="19"/>
       <c r="C21" s="12"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="48"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="51"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="77"/>
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
       <c r="N21" s="11"/>
@@ -3875,14 +3875,14 @@
       <c r="A22" s="18"/>
       <c r="B22" s="19"/>
       <c r="C22" s="12"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="23"/>
-      <c r="I22" s="24"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="24"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="50"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="49"/>
+      <c r="K22" s="51"/>
       <c r="L22" s="11"/>
       <c r="M22" s="11"/>
       <c r="N22" s="11"/>
@@ -3892,14 +3892,14 @@
       <c r="A23" s="18"/>
       <c r="B23" s="19"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="24"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="50"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="51"/>
       <c r="L23" s="11"/>
       <c r="M23" s="11"/>
       <c r="N23" s="11"/>
@@ -3909,14 +3909,14 @@
       <c r="A24" s="18"/>
       <c r="B24" s="19"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="23"/>
-      <c r="I24" s="24"/>
-      <c r="J24" s="22"/>
-      <c r="K24" s="48"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="77"/>
       <c r="L24" s="11"/>
       <c r="M24" s="11"/>
       <c r="N24" s="11"/>
@@ -3926,33 +3926,33 @@
       <c r="A25" s="18"/>
       <c r="B25" s="19"/>
       <c r="C25" s="12"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="27"/>
-      <c r="K25" s="29"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="79"/>
+      <c r="I25" s="80"/>
+      <c r="J25" s="78"/>
+      <c r="K25" s="80"/>
       <c r="L25" s="11"/>
       <c r="M25" s="11"/>
       <c r="N25" s="11"/>
       <c r="O25" s="13"/>
     </row>
     <row r="26" spans="1:15" ht="27.5" customHeight="1" thickBot="1">
-      <c r="A26" s="33" t="s">
+      <c r="A26" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="35"/>
+      <c r="B26" s="88"/>
+      <c r="C26" s="88"/>
+      <c r="D26" s="88"/>
+      <c r="E26" s="88"/>
+      <c r="F26" s="88"/>
+      <c r="G26" s="88"/>
+      <c r="H26" s="88"/>
+      <c r="I26" s="88"/>
+      <c r="J26" s="88"/>
+      <c r="K26" s="89"/>
       <c r="L26" s="14">
         <f>SUM(L9:L25)</f>
         <v>0</v>
@@ -3971,112 +3971,169 @@
       </c>
     </row>
     <row r="27" spans="1:15" ht="96" customHeight="1" thickBot="1">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="90" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="39" t="s">
+      <c r="B27" s="91"/>
+      <c r="C27" s="92"/>
+      <c r="D27" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="40"/>
-      <c r="J27" s="40"/>
-      <c r="K27" s="40"/>
-      <c r="L27" s="40"/>
-      <c r="M27" s="40"/>
-      <c r="N27" s="40"/>
-      <c r="O27" s="41"/>
+      <c r="E27" s="94"/>
+      <c r="F27" s="94"/>
+      <c r="G27" s="94"/>
+      <c r="H27" s="94"/>
+      <c r="I27" s="94"/>
+      <c r="J27" s="94"/>
+      <c r="K27" s="94"/>
+      <c r="L27" s="94"/>
+      <c r="M27" s="94"/>
+      <c r="N27" s="94"/>
+      <c r="O27" s="95"/>
     </row>
     <row r="28" spans="1:15" ht="57.5" customHeight="1">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="96" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="43"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="43"/>
-      <c r="I28" s="43"/>
-      <c r="J28" s="43"/>
-      <c r="K28" s="43"/>
-      <c r="L28" s="43"/>
-      <c r="M28" s="43"/>
-      <c r="N28" s="43"/>
-      <c r="O28" s="44"/>
+      <c r="B28" s="97"/>
+      <c r="C28" s="97"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="97"/>
+      <c r="G28" s="97"/>
+      <c r="H28" s="97"/>
+      <c r="I28" s="97"/>
+      <c r="J28" s="97"/>
+      <c r="K28" s="97"/>
+      <c r="L28" s="97"/>
+      <c r="M28" s="97"/>
+      <c r="N28" s="97"/>
+      <c r="O28" s="98"/>
     </row>
     <row r="29" spans="1:15" ht="76.25" customHeight="1">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="99" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="46"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46"/>
-      <c r="H29" s="46"/>
-      <c r="I29" s="46"/>
-      <c r="J29" s="46"/>
-      <c r="K29" s="46"/>
-      <c r="L29" s="46"/>
-      <c r="M29" s="46"/>
-      <c r="N29" s="46"/>
-      <c r="O29" s="47"/>
+      <c r="B29" s="100"/>
+      <c r="C29" s="100"/>
+      <c r="D29" s="100"/>
+      <c r="E29" s="100"/>
+      <c r="F29" s="100"/>
+      <c r="G29" s="100"/>
+      <c r="H29" s="100"/>
+      <c r="I29" s="100"/>
+      <c r="J29" s="100"/>
+      <c r="K29" s="100"/>
+      <c r="L29" s="100"/>
+      <c r="M29" s="100"/>
+      <c r="N29" s="100"/>
+      <c r="O29" s="101"/>
     </row>
     <row r="30" spans="1:15" ht="65" customHeight="1">
-      <c r="A30" s="45" t="s">
+      <c r="A30" s="99" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="46"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="46"/>
-      <c r="J30" s="46"/>
-      <c r="K30" s="46"/>
-      <c r="L30" s="46"/>
-      <c r="M30" s="46"/>
-      <c r="N30" s="46"/>
-      <c r="O30" s="47"/>
+      <c r="B30" s="100"/>
+      <c r="C30" s="100"/>
+      <c r="D30" s="100"/>
+      <c r="E30" s="100"/>
+      <c r="F30" s="100"/>
+      <c r="G30" s="100"/>
+      <c r="H30" s="100"/>
+      <c r="I30" s="100"/>
+      <c r="J30" s="100"/>
+      <c r="K30" s="100"/>
+      <c r="L30" s="100"/>
+      <c r="M30" s="100"/>
+      <c r="N30" s="100"/>
+      <c r="O30" s="101"/>
     </row>
     <row r="31" spans="1:15" ht="22.25" customHeight="1" thickBot="1">
-      <c r="A31" s="30"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
-      <c r="J31" s="31"/>
-      <c r="K31" s="31"/>
-      <c r="L31" s="31"/>
-      <c r="M31" s="31"/>
-      <c r="N31" s="31"/>
-      <c r="O31" s="32"/>
+      <c r="A31" s="84"/>
+      <c r="B31" s="85"/>
+      <c r="C31" s="85"/>
+      <c r="D31" s="85"/>
+      <c r="E31" s="85"/>
+      <c r="F31" s="85"/>
+      <c r="G31" s="85"/>
+      <c r="H31" s="85"/>
+      <c r="I31" s="85"/>
+      <c r="J31" s="85"/>
+      <c r="K31" s="85"/>
+      <c r="L31" s="85"/>
+      <c r="M31" s="85"/>
+      <c r="N31" s="85"/>
+      <c r="O31" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="93">
-    <mergeCell ref="A31:O31"/>
-    <mergeCell ref="A26:K26"/>
-    <mergeCell ref="A28:O28"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="D27:O27"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="A29:O29"/>
-    <mergeCell ref="A30:O30"/>
+    <mergeCell ref="L4:O4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:O5"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L3:O3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:O2"/>
+    <mergeCell ref="A4:C5"/>
+    <mergeCell ref="D4:E5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G18:I18"/>
     <mergeCell ref="L6:O6"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="D9:F9"/>
@@ -4093,73 +4150,16 @@
     <mergeCell ref="D13:F13"/>
     <mergeCell ref="L7:O7"/>
     <mergeCell ref="D8:F8"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="A4:C5"/>
-    <mergeCell ref="D4:E5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:O2"/>
-    <mergeCell ref="L3:O3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="L4:O4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:O5"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="A29:O29"/>
+    <mergeCell ref="A30:O30"/>
+    <mergeCell ref="A31:O31"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A28:O28"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:O27"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">

</xml_diff>